<commit_message>
feat: add card-validations test script, bizagi cancel flow and gitignore
- card_validations_test.py: prueba POST card-validations con subprocess curl, API key leida desde token.txt
- bizagi_cancel_case.py: cancela caso desde la UI de Bizagi (Admin) sin requerir token
- cancel_case_workflow.py: cancela caso via endpoint cancel-request usando token
- bizagi_automator.py: mejoras en flujo de consulta
- test_cases.json + test_cases.xlsx: 8 casos agrupados para card-validations
- .gitignore: excluye token.txt, __pycache__, evidences/ y archivos .env
- CLAUDE.md: nuevos PROMPTS 5-8 y endpoints de feature flags independientes
- workflows: cancelar_caso, cancelar_caso_vigente, consultar_pr

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -508,7 +508,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>TC001 - Thank You Page muestra mensaje correcto para Reactivación de cupo</t>
+          <t>TC001 - Flags ON: códigos de Reactivación (O, V, I, W) permiten el paso con tipoSolicitud 3</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -530,10 +530,14 @@
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Precondiciones:
-- Usuario autenticado en el flujo autogestionado
-- Solicitud de Reactivación de cupo procesada exitosamente en Bizagi
-- noveltyType = 3 enviado por WebSocket al Frontend
-- Variante de Reactivación configurada en Drupal</t>
+- Flag Reactivación: true
+- Flag Incremento: true (cualquier valor)
+- Usuarios con códigos de Reactivación en bolsillo 31 y tarjetaAmparada: false
+  · CC 52526685 → código O (CUPO CONGELADO)
+  · CC 51760693 → código V (CUENTA DEVOLUCION VOLUNTARIA)
+  · CC 41336668 → código V (CUENTA DEVOLUCION VOLUNTARIA)
+  · CC 79528108 → código I (INACTIVO)
+  · Pendiente dato → código W</t>
         </is>
       </c>
       <c r="F3" s="3" t="n"/>
@@ -544,7 +548,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Given que el usuario completó el flujo de Reactivación de cupo</t>
+          <t>Given que los usuarios anteriores inician solicitud de crédito con flag Reactivación activo</t>
         </is>
       </c>
       <c r="F4" s="3" t="n"/>
@@ -555,7 +559,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>When el sistema redirige al usuario a la Thank You Page</t>
+          <t>When se consume POST /loans/eligibility/internal/v1/card-validations para cada usuario con tipo CO1C</t>
         </is>
       </c>
       <c r="F5" s="3" t="n"/>
@@ -566,12 +570,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Then la página debe mostrar el mensaje de solicitud en proceso</t>
+          <t>Then la respuesta HTTP es 200 para todos</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Se muestra el mensaje: 'Tu solicitud ha sido recibida. Te notificaremos cuando tu cupo esté activo'</t>
+          <t>HTTP 200</t>
         </is>
       </c>
     </row>
@@ -581,587 +585,1011 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>And el mensaje NO debe indicar que el cupo está disponible de inmediato</t>
+          <t>And el campo estado es OK para todos</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>No aparece ningún texto como 'Tu cupo está listo' o 'Ya puedes usar tu cupo'</t>
+          <t>"estado": "OK"</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>TC002 - Thank You Page de Originación NO se ve afectada por el cambio</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Ecosistema Digital Crédito y Seguros</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>And el campo tipoSolicitud es 3 para todos (códigos O, V, I, W)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>"tipoSolicitud": 3</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="D9" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Precondiciones:
-- Usuario autenticado en el flujo autogestionado
-- Solicitud de Originación (cupo nuevo) procesada exitosamente
-- noveltyType = 1 enviado por WebSocket al Frontend</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="n"/>
+          <t>And el campo tarjetaAmparada es false para todos</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>"tarjetaAmparada": false</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="D10" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Given que el usuario completó el flujo de Originación de crédito</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="n"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>TC002 - Flags ON: códigos de Incremento (1, N, S) permiten el paso con tipoSolicitud 2</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Ecosistema Digital Crédito y Seguros</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="D11" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>When el sistema redirige al usuario a la Thank You Page</t>
+          <t>Precondiciones:
+- Flag Reactivación: true (cualquier valor)
+- Flag Incremento: true
+- Usuarios con códigos de Incremento en bolsillo 31 y tarjetaAmparada: false
+  · CC 80810798   → código 1 (NORMAL)
+  · CC 1140814422 → código 1, tarjeta estado 7 (CAMBIO DE CLAVE OBLIGATORIO)
+  · CC 1097397286 → código 1, tarjeta estado S (SUSPENDIDO/SOBRECUPO)
+  · CC 52966724   → código 1, tarjeta estado 0 (PENDIENTE POR ACTIVAR)
+  · CC 1023876310 → código 1 (NORMAL)
+  · Pendiente dato → código N
+  · Pendiente dato → código S</t>
         </is>
       </c>
       <c r="F11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="D12" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Then debe mostrarse el mensaje original de Originación sin modificaciones</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>El mensaje mostrado es el existente para Originación, sin cambios respecto al comportamiento anterior</t>
-        </is>
-      </c>
+          <t>Given que los usuarios anteriores inician solicitud de crédito con flag Incremento activo</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="D13" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>And NO se muestra el mensaje de novedades asíncronas</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>No aparece el texto 'Te notificaremos cuando tu cupo esté activo'</t>
-        </is>
-      </c>
+          <t>When se consume POST /loans/eligibility/internal/v1/card-validations para cada usuario con tipo CO1C</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>TC003 - Mensaje de Reactivación es diferente al mensaje de Originación</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Ecosistema Digital Crédito y Seguros</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Then la respuesta HTTP es 200 para todos</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 200</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="D15" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Precondiciones:
-- Acceso a dos sesiones: una con flujo de Originación y otra con flujo de Reactivación
-- Ambas solicitudes procesadas exitosamente</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="n"/>
+          <t>And el campo estado es OK para todos</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>"estado": "OK"</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="D16" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Given que se tienen dos Thank You Pages cargadas: una de Originación y una de Reactivación</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="n"/>
+          <t>And el campo tipoSolicitud es 2 para todos (códigos 1, N, S)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>"tipoSolicitud": 2</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="D17" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>When se compara el contenido de ambas páginas</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="n"/>
+          <t>And el campo tarjetaAmparada es false para todos</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>"tarjetaAmparada": false</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="D18" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Then los mensajes deben ser distintos entre sí</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>La Thank You Page de Reactivación muestra un mensaje diferente al de Originación</t>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>TC003 - Flags OFF: códigos de Reactivación e Incremento son bloqueados</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Ecosistema Digital Crédito y Seguros</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>TC004 - Thank You Page carga correctamente el mensaje desde Drupal para Reactivación</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Ecosistema Digital Crédito y Seguros</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
+      <c r="D19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Precondiciones:
+- Flag Reactivación: false
+- Flag Incremento: false
+- Usuarios con códigos de novedad
+  · CC 41336668 → código V (Reactivación)
+  · CC 79528108 → código I (Reactivación)
+  · CC 1140814422 → código 1 (Incremento)
+  · CC 80810798 → código 1 (Incremento)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="D20" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Precondiciones:
-- Variante de Reactivación configurada y publicada en Drupal
-- noveltyType = 3 disponible en el evento WebSocket</t>
+          <t>Given que los usuarios anteriores inician solicitud de crédito con ambas flags desactivadas</t>
         </is>
       </c>
       <c r="F20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="D21" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Given que el Frontend recibe noveltyType = 3 desde el WebSocket</t>
+          <t>When se consume POST /loans/eligibility/internal/v1/card-validations para cada usuario</t>
         </is>
       </c>
       <c r="F21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="D22" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>When el Frontend consulta el contenido correspondiente en Drupal</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="n"/>
+          <t>Then la respuesta HTTP es 200 para todos</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 200</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="D23" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Then se renderiza el contenido de la variante de Reactivación configurada en Drupal</t>
+          <t>And el campo estado es VALIDATION_ERROR para todos</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>El texto y los elementos visuales corresponden exactamente a la variante de Reactivación publicada en el CMS</t>
+          <t>"estado": "VALIDATION_ERROR"</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>TC005 - Pixel Perfect: Thank You Page de Reactivación coincide visualmente con el diseño de Figma</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Ecosistema Digital Crédito y Seguros</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Design</t>
+      <c r="D24" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>And el campo tipoSolicitud NO está presente en ninguna respuesta</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>tipoSolicitud ausente</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Precondiciones:
-- Diseño aprobado de la Thank You Page de Reactivación disponible en Figma (pantalla exportada como imagen de referencia)
-- Entorno de pruebas estable con la Thank You Page de Reactivación desplegada
-- Herramienta de comparación visual configurada (ej. Percy, Applitools o captura manual pixel-by-pixel)
-- noveltyType = 3 recibido correctamente por el Frontend</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="n"/>
+          <t>And el campo codigoErrorValidacion es INVALID_REQUIREMENTS para todos</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>"codigoErrorValidacion": "INVALID_REQUIREMENTS"</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="D26" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Given que la Thank You Page de Reactivación está renderizada en el navegador en resolución de escritorio (1440x900)</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="n"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>TC004 - Flags independientes: cada flag bloquea solo su tipo de novedad</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Ecosistema Digital Crédito y Seguros</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="D27" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>When se toma una captura de pantalla completa de la página y se compara pixel a pixel contra el diseño de referencia exportado de Figma</t>
+          <t>Precondiciones:
+- Escenario A: Flag Reactivación ON, Flag Incremento OFF
+  · CC 79528108 → código I (Reactivación) debe pasar
+  · CC 1140814422 → código 1 (Incremento) debe bloquearse
+- Escenario B: Flag Reactivación OFF, Flag Incremento ON
+  · CC 1140814422 → código 1 (Incremento) debe pasar
+  · CC 79528108 → código I (Reactivación) debe bloquearse</t>
         </is>
       </c>
       <c r="F27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="D28" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Then la diferencia visual entre la captura y el diseño de Figma debe ser igual a cero o inferior al umbral permitido (≤ 0.1%)</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>No existen diferencias visuales detectables: colores, tipografía, márgenes, espaciado e iconos coinciden exactamente con el diseño de Figma</t>
-        </is>
-      </c>
+          <t>Given escenario A: Flag Reactivación ON, Flag Incremento OFF</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="D29" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>And los elementos gráficos (logo, íconos, imágenes decorativas) se renderizan sin distorsión ni recorte</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Cada elemento visual ocupa la posición y dimensiones definidas en Figma sin desbordamientos ni desplazamientos</t>
-        </is>
-      </c>
+          <t>When se consume el servicio con CC 79528108 (código I)</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="D30" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>And la página es responsiva y mantiene la fidelidad visual en resolución móvil (375x812)</t>
+          <t>Then el estado es OK y tipoSolicitud es 3</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>La comparación pixel a pixel en vista móvil no supera el umbral permitido respecto al frame móvil de Figma</t>
+          <t>"estado": "OK", "tipoSolicitud": 3</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>TC006 - Fidelidad de contenido: textos y etiquetas de la Thank You Page de Reactivación coinciden con Figma</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>Ecosistema Digital Crédito y Seguros</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
+      <c r="D31" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>When se consume el servicio con CC 1140814422 (código 1)</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="D32" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Precondiciones:
-- Especificación de contenido de la Thank You Page de Reactivación documentada en Figma (títulos, cuerpo, botones, disclaimers)
-- noveltyType = 3 procesado exitosamente
-- Acceso a la Thank You Page de Reactivación en entorno de pruebas</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="n"/>
+          <t>Then el estado es VALIDATION_ERROR y tipoSolicitud ausente</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>"estado": "VALIDATION_ERROR", tipoSolicitud ausente</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="D33" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Given que la Thank You Page de Reactivación está visible para el usuario</t>
+          <t>Given escenario B: Flag Reactivación OFF, Flag Incremento ON</t>
         </is>
       </c>
       <c r="F33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="D34" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>When se revisa el título principal de la página</t>
+          <t>When se consume el servicio con CC 1140814422 (código 1)</t>
         </is>
       </c>
       <c r="F34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="D35" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Then el título debe coincidir exactamente con el texto definido en el diseño de Figma (mayúsculas, puntuación e idioma incluidos)</t>
+          <t>Then el estado es OK y tipoSolicitud es 2</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>El título mostrado es idéntico al especificado en Figma para la variante de Reactivación</t>
+          <t>"estado": "OK", "tipoSolicitud": 2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>And el cuerpo del mensaje (párrafo descriptivo) coincide con el texto de Figma sin palabras faltantes ni adicionales</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>El texto del cuerpo es exactamente el definido en Figma, sin truncamientos ni diferencias ortográficas</t>
-        </is>
-      </c>
+          <t>When se consume el servicio con CC 79528108 (código I)</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="D37" s="3" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>And las etiquetas de botones de acción (CTA) coinciden con el copy de Figma</t>
+          <t>Then el estado es VALIDATION_ERROR y tipoSolicitud ausente</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Cada botón muestra el texto de llamada a la acción especificado en Figma (ej. 'Ir al inicio', 'Ver mis productos')</t>
+          <t>"estado": "VALIDATION_ERROR", tipoSolicitud ausente</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="D38" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>And los textos de pie de página o disclaimers legales coinciden con el contenido de Figma</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Los disclaimers se muestran completos y sin variaciones respecto a lo definido en Figma</t>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>TC005 - tarjetaAmparada bloquea siempre independiente del flag y código Ascard</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Ecosistema Digital Crédito y Seguros</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>TC007 - El contenido de la Thank You Page de Reactivación proviene de Drupal y no está hardcodeado en el Frontend</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Ecosistema Digital Crédito y Seguros</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
+      <c r="D39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Precondiciones:
+- Flag Reactivación: true
+- Flag Incremento: true
+- Usuarios con tarjetaAmparada: true (tienen tarjeta tipo 6)
+  · CC 52634111 → código I (Reactivación), tarjetaAmparada: true
+  · CC 1095915781 → código I (Reactivación), tarjetaAmparada: true
+  · CC 1013595547 → código I (Reactivación), tarjetaAmparada: true
+  · CC 20156603 → código I (Reactivación), tarjetaAmparada: true</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="D40" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Precondiciones:
-- Acceso a la consola de red del navegador (DevTools → Network)
-- Variante de Reactivación publicada en Drupal con contenido conocido y verificable
-- noveltyType = 3 enviado por WebSocket
-- Segunda variante de prueba con contenido diferente disponible en Drupal (para validar dinamismo)</t>
+          <t>Given que los usuarios anteriores tienen tarjeta amparada tipo 6 e inician solicitud de crédito</t>
         </is>
       </c>
       <c r="F40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="D41" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Given que el Frontend recibe noveltyType = 3 y renderiza la Thank You Page de Reactivación</t>
+          <t>When se consume POST /loans/eligibility/internal/v1/card-validations para cada usuario con tipo CO1C</t>
         </is>
       </c>
       <c r="F41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="D42" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>When se inspecciona la pestaña Network en DevTools durante la carga de la página</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="n"/>
+          <t>Then la respuesta HTTP es 200 para todos</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 200</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="D43" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Then debe existir al menos una llamada HTTP al endpoint de Drupal que retorne el contenido de la variante de Reactivación</t>
+          <t>And el campo estado es VALIDATION_ERROR para todos aunque las flags estén activas</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Se registra una petición GET al CMS Drupal (ej. /jsonapi/ o /api/... ) con respuesta 200 que incluye los textos mostrados en pantalla</t>
+          <t>"estado": "VALIDATION_ERROR"</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="D44" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>And el contenido visible en pantalla corresponde al payload devuelto por Drupal y no a cadenas de texto definidas en el código fuente del Frontend</t>
+          <t>And el campo tarjetaAmparada es true para todos</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Los textos de título, cuerpo y botones de la Thank You Page coinciden exactamente con los campos del JSON retornado por Drupal</t>
+          <t>"tarjetaAmparada": true</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="D45" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>And el campo tipoSolicitud NO está presente en ninguna respuesta</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>tipoSolicitud ausente</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>TC006 - Códigos Ascard desconocidos/mora bloquean siempre con ambas flags ON</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Ecosistema Digital Crédito y Seguros</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="D47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Precondiciones:
+- Flag Reactivación: true
+- Flag Incremento: true
+- Usuarios con códigos fuera de los sets de novedad
+  · CC 79584194 → código R (CUENTA REFINANCIADA)
+  · CC 19184974 → código K (CUENTA CASTIGADA)
+  · CC 19246507 → código J (CUENTA EN COBRO PRE JURIDICO)
+  · CC 11259747 → código J (CUENTA EN COBRO PRE JURIDICO)
+  · CC 547911   → código B (CUENTA CANCELADA POR EL BANCO)
+  · CC 1023944601 → código Y (COBRO JURIDICO)
+  · CC 13617086 → código A (POR MORA EN SUS PRODUCTOS)</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="n"/>
+    </row>
+    <row r="48">
+      <c r="D48" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Given que los usuarios anteriores inician solicitud de crédito</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="D49" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>When se consume POST /loans/eligibility/internal/v1/card-validations para cada usuario con tipo CO1C</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="n"/>
+    </row>
+    <row r="50">
+      <c r="D50" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Then la respuesta HTTP es 200 para todos</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="D51" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>And el campo estado es VALIDATION_ERROR para todos</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>"estado": "VALIDATION_ERROR"</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="D52" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>When se modifica el contenido de la variante de Reactivación directamente en Drupal (sin despliegue de Frontend) y se recarga la Thank You Page</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="n"/>
-    </row>
-    <row r="46">
-      <c r="D46" s="3" t="n">
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>And el campo tipoSolicitud NO está presente en ninguna respuesta</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>tipoSolicitud ausente</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="D53" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>Then la página muestra el contenido actualizado de Drupal sin necesidad de un nuevo despliegue del Frontend</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>El cambio de contenido en Drupal se refleja de forma inmediata en la Thank You Page, confirmando que la fuente de verdad es el CMS</t>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>And el campo codigoErrorValidacion es INVALID_REQUIREMENTS para todos</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>"codigoErrorValidacion": "INVALID_REQUIREMENTS"</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>TC007 - Sin tarjeta activa y tipo documento CE mapeado a CO1E</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Ecosistema Digital Crédito y Seguros</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="D55" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Precondiciones:
+- Flag Reactivación: true
+- Flag Incremento: true
+- Escenario A: usuarios sin tarjeta multiservicios activa
+  · CC 80833648, CC 382429, CC 1024539415 → dataTarjeta vacío
+- Escenario B: usuario CE 382429
+  · El tipo CE debe enviarse como CO1E en el body (no como CE, genera HTTP 400)</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n"/>
+    </row>
+    <row r="56">
+      <c r="D56" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Given escenario A: usuarios sin tarjeta activa</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="n"/>
+    </row>
+    <row r="57">
+      <c r="D57" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>When se consume POST /loans/eligibility/internal/v1/card-validations con tipo CO1C para CC 80833648, CC 382429, CC 1024539415</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="D58" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Then la respuesta HTTP es 200 para todos</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="D59" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>And el campo codigoErrorValidacion es CARD_STATUS</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>"codigoErrorValidacion": "CARD_STATUS"</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="D60" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>And el campo reglaErrorValidacion es Tarjeta multiservicios no activa</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>"reglaErrorValidacion": "Tarjeta multiservicios no activa"</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="D61" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Given escenario B: usuario CE 382429</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="n"/>
+    </row>
+    <row r="62">
+      <c r="D62" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>When se consume el servicio con body {"documento": {"tipo": "CO1E", "numero": "382429"}}</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n"/>
+    </row>
+    <row r="63">
+      <c r="D63" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Then la respuesta HTTP es 200 (no 400 — el 400 ocurre si se envía tipo CE en lugar de CO1E)</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>HTTP 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="D64" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>And el campo codigoErrorValidacion es CARD_STATUS</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>"codigoErrorValidacion": "CARD_STATUS"</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>TC008 - Regresión: tipoSolicitud presente en OK, ausente en VALIDATION_ERROR</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Ecosistema Digital Crédito y Seguros</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="D66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Precondiciones:
+- Flag Reactivación: true
+- Flag Incremento: true
+- Usuarios OK: CC 52526685 (Reactivación), CC 80810798 (Incremento)
+- Usuarios VALIDATION_ERROR: CC 19184974 (K), CC 79584194 (R), CC 52634111 (tarjetaAmparada)</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="D67" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Given que se consumen usuarios que generan estado OK y usuarios que generan VALIDATION_ERROR</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="n"/>
+    </row>
+    <row r="68">
+      <c r="D68" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>When se revisan todas las respuestas OK</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n"/>
+    </row>
+    <row r="69">
+      <c r="D69" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Then el campo tipoSolicitud SIEMPRE está presente en respuestas con estado OK</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>tipoSolicitud presente</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="D70" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>And tipoSolicitud es 3 para códigos de Reactivación (O, V, I, W)</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>"tipoSolicitud": 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="D71" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>And tipoSolicitud es 2 para códigos de Incremento (1, N, S)</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>"tipoSolicitud": 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="D72" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>When se revisan todas las respuestas VALIDATION_ERROR</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="n"/>
+    </row>
+    <row r="73">
+      <c r="D73" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Then el campo tipoSolicitud NUNCA está presente en respuestas con estado VALIDATION_ERROR</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>tipoSolicitud ausente en toda respuesta VALIDATION_ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="D74" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>And el campo datosError siempre está presente con codigoErrorValidacion y reglaErrorValidacion</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>datosError presente</t>
         </is>
       </c>
     </row>

</xml_diff>